<commit_message>
Block ALL actions for the first 15 seconds after entry to avoid spread-induced stop loss
</commit_message>
<xml_diff>
--- a/reports/Daily_Report_2026-05-25.xlsx
+++ b/reports/Daily_Report_2026-05-25.xlsx
@@ -515,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -527,7 +527,7 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -541,7 +541,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated on 2026-05-25 22:29:09 IST</t>
+          <t>Generated on 2026-05-25 22:32:45 IST</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>18.08781376922316</v>
+        <v>18.12196658913581</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>1501.288542845523</v>
+        <v>1504.123226898272</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -603,7 +603,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>58.65%</t>
+          <t>58.73%</t>
         </is>
       </c>
     </row>
@@ -741,75 +741,120 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-25T22:32:41.507541+05:30</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-25T22:32:45.291124+05:30</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>C-BTC-78600-260526</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>93.58507857754148</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>96.56591974</v>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>P-BTC-77000-260526</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="n">
+        <v>88.44500606158498</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>85.1226367</v>
+      </c>
+      <c r="I16" s="10" t="n">
+        <v>18.20300846391265</v>
+      </c>
+      <c r="J16" s="11" t="n">
+        <v>0.03415281991264862</v>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>EOD Square-off</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Risk &amp; Market Metrics</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Daily Loss Limit Hit</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>SL Hits</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="n">
-        <v>0</v>
+          <t>Daily Loss Limit Hit</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Hedging Activity</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+          <t>SL Hits</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>ADX Value</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="n">
-        <v>0</v>
+          <t>Hedging Activity</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>IV Level</t>
-        </is>
-      </c>
-      <c r="B22" s="13" t="n">
-        <v>0.413335260904325</v>
+          <t>ADX Value</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
+          <t>IV Level</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="n">
+        <v>0.4139179401310616</v>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
           <t>High Impact News</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>None</t>
         </is>

</xml_diff>

<commit_message>
Fix start_ts NoneType bug in loop
</commit_message>
<xml_diff>
--- a/reports/Daily_Report_2026-05-25.xlsx
+++ b/reports/Daily_Report_2026-05-25.xlsx
@@ -515,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated on 2026-05-25 22:32:45 IST</t>
+          <t>Generated on 2026-05-25 22:40:22 IST</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>18.12196658913581</v>
+        <v>36.22956175467251</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>1504.123226898272</v>
+        <v>3007.053625637818</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -603,7 +603,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>58.73%</t>
+          <t>58.65%</t>
         </is>
       </c>
     </row>
@@ -786,75 +786,120 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-25T22:40:17.423707+05:30</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-25T22:40:21.827394+05:30</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>C-BTC-78600-260526</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>89.13674788440676</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>87.67965089</v>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>P-BTC-77000-260526</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="n">
+        <v>94.64925927096023</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>94.33618993</v>
+      </c>
+      <c r="I17" s="10" t="n">
+        <v>18.3786007155367</v>
+      </c>
+      <c r="J17" s="11" t="n">
+        <v>18.1075951655367</v>
+      </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>EOD Square-off</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Risk &amp; Market Metrics</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Daily Loss Limit Hit</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>SL Hits</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="n">
-        <v>0</v>
+          <t>Daily Loss Limit Hit</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Hedging Activity</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+          <t>SL Hits</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>ADX Value</t>
-        </is>
-      </c>
-      <c r="B22" s="12" t="n">
-        <v>0</v>
+          <t>Hedging Activity</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>IV Level</t>
-        </is>
-      </c>
-      <c r="B23" s="13" t="n">
-        <v>0.4139179401310616</v>
+          <t>ADX Value</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
+          <t>IV Level</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>0.4141503042726081</v>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
           <t>High Impact News</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>None</t>
         </is>

</xml_diff>

<commit_message>
Enhance Smart Hedging: Dynamic SL, Loss-based Activation, and PnL Tracking
</commit_message>
<xml_diff>
--- a/reports/Daily_Report_2026-05-25.xlsx
+++ b/reports/Daily_Report_2026-05-25.xlsx
@@ -515,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated on 2026-05-25 22:40:22 IST</t>
+          <t>Generated on 2026-05-25 22:56:16 IST</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>36.22956175467251</v>
+        <v>46.05135055563546</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>3007.053625637818</v>
+        <v>3822.262096117743</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
@@ -603,7 +603,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>58.65%</t>
+          <t>58.69%</t>
         </is>
       </c>
     </row>
@@ -831,75 +831,120 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-25T22:56:15.395202+05:30</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-25T22:56:16.318519+05:30</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>C-BTC-78400-260526</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>98.1068114717429</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>98.1068114717429</v>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>P-BTC-76800-260526</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>87.86699094788658</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>86.40383125</v>
+      </c>
+      <c r="I18" s="10" t="n">
+        <v>18.59738024196295</v>
+      </c>
+      <c r="J18" s="11" t="n">
+        <v>9.821788800962949</v>
+      </c>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>EOD Square-off</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Risk &amp; Market Metrics</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Daily Loss Limit Hit</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>SL Hits</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="n">
-        <v>0</v>
+          <t>Daily Loss Limit Hit</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Hedging Activity</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+          <t>SL Hits</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>ADX Value</t>
-        </is>
-      </c>
-      <c r="B23" s="12" t="n">
-        <v>0</v>
+          <t>Hedging Activity</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>IV Level</t>
-        </is>
-      </c>
-      <c r="B24" s="13" t="n">
-        <v>0.4141503042726081</v>
+          <t>ADX Value</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
+          <t>IV Level</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="n">
+        <v>0.4130171852031455</v>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
           <t>High Impact News</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>None</t>
         </is>

</xml_diff>